<commit_message>
Create accounting cash flow analyzer with full file audit
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/monthly_cash_flow_reconstruction.xlsx
+++ b/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/monthly_cash_flow_reconstruction.xlsx
@@ -23,77 +23,77 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>revenue_if_available</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>payroll_brutto</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>payroll_netto</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>health_insurance_due</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>health_insurance_paid</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>health_insurance_unpaid</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tax_due</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>tax_paid</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>tax_unpaid</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>operating_costs_due</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>operating_costs_paid</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>operating_costs_unpaid</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>total_monthly_obligations</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>total_paid</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>total_unpaid</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>first_visible_financial_pressure_yes_no</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
@@ -125,22 +125,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t/>
+          <t>517.65</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>137896.85</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t/>
+          <t>435.00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t/>
+          <t>21.02</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -150,22 +150,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t/>
+          <t>19.00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t/>
+          <t>1.77</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t/>
+          <t>141002.75</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -175,32 +175,32 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t/>
+          <t>141974.40</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t/>
+          <t>137919.64</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -222,22 +222,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t/>
+          <t>10500.10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>11056.17</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t/>
+          <t>991.96</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t/>
+          <t>833.58</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -247,22 +247,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t/>
+          <t>10531.34</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t/>
+          <t>821.97</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t/>
+          <t>53.04</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t/>
+          <t>826140081.04</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -272,32 +272,32 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t/>
+          <t>53.04</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t/>
+          <t>826162104.44</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t/>
+          <t>12711.72</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>106.08</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -324,7 +324,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -344,22 +344,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t/>
+          <t>19.00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t/>
+          <t>1.77</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t/>
+          <t>30.04</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -369,32 +369,32 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t/>
+          <t>49.04</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t/>
+          <t>20.77</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -421,7 +421,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t/>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -441,22 +441,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t/>
+          <t>19.00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t/>
+          <t>1.77</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t/>
+          <t>30.05</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -466,32 +466,32 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t/>
+          <t>49.05</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t/>
+          <t>20.77</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>38.00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -635,22 +635,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t/>
+          <t>38.00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t/>
+          <t>3.54</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t/>
+          <t>60.13</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -660,32 +660,32 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t/>
+          <t>98.13</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t/>
+          <t>41.54</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>80.00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t/>
+          <t>151148.76</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -732,22 +732,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t/>
+          <t>32.12</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t/>
+          <t>1.77</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t/>
+          <t>27.09</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t/>
+          <t>23175.77</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -757,32 +757,32 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t/>
+          <t>27.09</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t/>
+          <t>23207.89</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t/>
+          <t>151150.53</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>54.18</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -869,17 +869,17 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -906,17 +906,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t/>
+          <t>148369.66</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t/>
+          <t>88.53</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t/>
+          <t>15451.27</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -926,57 +926,57 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t/>
+          <t>5901.32</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t/>
+          <t>1.77</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t/>
+          <t>39.11</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t/>
+          <t>40907.07</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t/>
+          <t>37.18</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t/>
+          <t>39.11</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t/>
+          <t>46896.92</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t/>
+          <t>163859.88</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>78.22</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1003,17 +1003,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t/>
+          <t>166852.66</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t/>
+          <t>702400.72</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t/>
+          <t>516.00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1023,57 +1023,57 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t/>
+          <t>702445.44</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t/>
+          <t>517.77</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t/>
+          <t>40.20</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t/>
+          <t>769745.06</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t/>
+          <t>516.00</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t/>
+          <t>40.20</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t/>
+          <t>2174591.22</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t/>
+          <t>168402.43</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>80.40</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>195244.85</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1120,57 +1120,57 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t/>
+          <t>6434.68</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t/>
+          <t>16.88</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t/>
+          <t>67.19</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t/>
+          <t>95755.41</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t/>
+          <t>15.11</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t/>
+          <t>67.19</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t/>
+          <t>102190.09</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t/>
+          <t>195276.84</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>134.38</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1192,17 +1192,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t/>
+          <t>11062.00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t/>
+          <t>180268.79</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t/>
+          <t>7.09</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1217,22 +1217,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t/>
+          <t>11075.34</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t/>
+          <t>17.00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t/>
+          <t>34.03</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t/>
+          <t>34519.54</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1242,32 +1242,32 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t/>
+          <t>34.03</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t/>
+          <t>56663.97</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t/>
+          <t>180285.79</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>68.06</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>159310.00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t/>
+          <t>13.34</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1324,12 +1324,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t/>
+          <t>14.03</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t/>
+          <t>24239.62</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1339,32 +1339,32 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t/>
+          <t>14.03</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t/>
+          <t>24252.96</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t/>
+          <t>159310.00</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>28.06</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>143204.08</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t/>
+          <t>13649.05</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1411,57 +1411,57 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t/>
+          <t>19.00</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t/>
+          <t>13650.93</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t/>
+          <t>206.30</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t/>
+          <t>13649.05</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t/>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t/>
+          <t>225.30</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t/>
+          <t>184153.11</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1488,17 +1488,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t/>
+          <t>171721.61</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t/>
+          <t>167412.67</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t/>
+          <t>181061.72</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t/>
+          <t>13649.05</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t/>
+          <t>4268.37</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t/>
+          <t>13649.05</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1538,27 +1538,27 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t/>
+          <t>171681.04</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t/>
+          <t>380081.43</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t/>
+          <t>153436.60</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t/>
+          <t>872.35</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1635,27 +1635,27 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t/>
+          <t>872.35</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t/>
+          <t>153436.60</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t/>
+          <t>102207.65</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t/>
+          <t>2497.56</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1732,27 +1732,27 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t/>
+          <t>2497.56</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t/>
+          <t>102207.65</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>54103.70</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t/>
+          <t>12030.37</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1829,27 +1829,27 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t/>
+          <t>12030.37</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t/>
+          <t>54103.70</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>No extracted accounting values for this month.</t>
+          <t/>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve accounting extraction accuracy after validation
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/monthly_cash_flow_reconstruction.xlsx
+++ b/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/monthly_cash_flow_reconstruction.xlsx
@@ -125,22 +125,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>517.65</t>
+          <t/>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>137896.85</t>
+          <t/>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>58321.97</t>
+          <t/>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>12505.81</t>
+          <t/>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -150,12 +150,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>57905.97</t>
+          <t>268.68</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12486.56</t>
+          <t>83428.40</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -165,12 +165,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>146827.86</t>
+          <t>163577.00</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>12469.77</t>
+          <t/>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -180,12 +180,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>263573.45</t>
+          <t>163845.68</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>175358.99</t>
+          <t>83428.40</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -222,22 +222,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10500.10</t>
+          <t/>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>11037.17</t>
+          <t/>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>59425.27</t>
+          <t/>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>8119.23</t>
+          <t/>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -247,47 +247,47 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68107.32</t>
+          <t>11182.78</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>8105.85</t>
+          <t>84182.26</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>33.04</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>826145216.37</t>
+          <t>659.11</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>7277.62</t>
+          <t/>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>33.04</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>826283249.06</t>
+          <t>11841.89</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>34539.87</t>
+          <t>84182.26</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>66.08</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -324,17 +324,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>19.00</t>
+          <t/>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>53716.12</t>
+          <t/>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6568.57</t>
+          <t/>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -344,12 +344,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>53735.12</t>
+          <t>2432.55</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>6570.34</t>
+          <t>60336.62</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -359,12 +359,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>4775.75</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>6556.53</t>
+          <t/>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -374,12 +374,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>112226.99</t>
+          <t>2452.55</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>19714.44</t>
+          <t>60336.62</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -421,17 +421,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19.00</t>
+          <t/>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>51583.91</t>
+          <t/>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7245.07</t>
+          <t/>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -441,12 +441,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>51602.91</t>
+          <t>363.00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5698.84</t>
+          <t>80205.88</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -456,12 +456,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>4069.27</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>7237.02</t>
+          <t/>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>107256.09</t>
+          <t>383.00</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>20199.93</t>
+          <t>80205.88</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -518,47 +518,47 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.00</t>
+          <t/>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>54457.03</t>
+          <t/>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5881.24</t>
+          <t>-216.63</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t/>
+          <t>68848.69</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>54475.02</t>
+          <t>435.13</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>5883.01</t>
+          <t>71122.06</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>20.00</t>
+          <t>68868.69</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>4064.50</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>5890.28</t>
+          <t/>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -568,17 +568,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>112996.55</t>
+          <t>455.13</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>17673.53</t>
+          <t>70905.43</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>40.00</t>
+          <t>137737.38</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>19.00</t>
+          <t/>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>54779.05</t>
+          <t/>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6003.35</t>
+          <t/>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>54797.04</t>
+          <t>1137.00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>6005.12</t>
+          <t>84326.62</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>3031.10</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>5991.28</t>
+          <t/>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>112607.19</t>
+          <t>1157.00</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>18018.75</t>
+          <t>84326.62</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -712,17 +712,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>151148.76</t>
+          <t/>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>48872.69</t>
+          <t/>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7994.75</t>
+          <t>915.48</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -732,47 +732,47 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>48903.74</t>
+          <t>1267.39</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>7081.04</t>
+          <t>76420.25</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>27.09</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>25234.65</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>7985.67</t>
+          <t/>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>27.09</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>123011.08</t>
+          <t>1287.39</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>174210.22</t>
+          <t>77335.73</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>54.18</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -809,17 +809,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>19.00</t>
+          <t/>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>53051.12</t>
+          <t/>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>8563.49</t>
+          <t/>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>53070.12</t>
+          <t>2515.77</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>8565.26</t>
+          <t>59703.77</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2500.84</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>8550.40</t>
+          <t/>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>108622.08</t>
+          <t>2535.77</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>25698.15</t>
+          <t>59703.77</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -906,17 +906,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>148350.66</t>
+          <t/>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>21727.98</t>
+          <t/>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>26916.23</t>
+          <t/>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -926,47 +926,47 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3781.62</t>
+          <t/>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>11454.86</t>
+          <t>27518.62</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>19.11</t>
+          <t/>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>43726.68</t>
+          <t>303.00</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>11492.04</t>
+          <t/>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>19.11</t>
+          <t/>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>69236.28</t>
+          <t>303.00</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>198213.79</t>
+          <t>27518.62</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>38.22</t>
+          <t/>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1003,17 +1003,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>166852.66</t>
+          <t/>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>704413.94</t>
+          <t/>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>6902.07</t>
+          <t/>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1023,47 +1023,47 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>704458.66</t>
+          <t>1260.94</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>6903.84</t>
+          <t>32235.47</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>40.20</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>819894.22</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>6890.96</t>
+          <t/>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>40.20</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2228766.82</t>
+          <t>1280.94</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>187549.53</t>
+          <t>32235.47</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>80.40</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>195244.85</t>
+          <t/>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6457.35</t>
+          <t/>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>8348.14</t>
+          <t>1165.16</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1120,47 +1120,47 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3733.22</t>
+          <t>202.33</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>7173.64</t>
+          <t>36397.47</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>67.19</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>162033.09</t>
+          <t>18555.34</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>8326.91</t>
+          <t/>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>67.19</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>172223.66</t>
+          <t>18757.67</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>219093.54</t>
+          <t>37562.63</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>134.38</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>169225.79</t>
+          <t/>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>5924.52</t>
+          <t/>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7079.18</t>
+          <t/>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1217,47 +1217,47 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>4837.79</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>7070.83</t>
+          <t>25280.51</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>34.03</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>111540.78</t>
+          <t>17882.56</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>7054.05</t>
+          <t/>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>34.03</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>122303.09</t>
+          <t>17901.56</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>190429.85</t>
+          <t>25280.51</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>68.06</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1294,17 +1294,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>159310.00</t>
+          <t/>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2356.77</t>
+          <t/>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5718.89</t>
+          <t/>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1314,47 +1314,47 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1258.13</t>
+          <t/>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5703.88</t>
+          <t>25375.10</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>14.03</t>
+          <t/>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>92243.09</t>
+          <t>18938.06</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>5692.86</t>
+          <t/>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>14.03</t>
+          <t/>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>95857.99</t>
+          <t>18938.06</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>176425.63</t>
+          <t>25375.10</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>28.06</t>
+          <t/>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1391,17 +1391,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>143185.08</t>
+          <t/>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5758.30</t>
+          <t/>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>18651.96</t>
+          <t/>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4680.36</t>
+          <t/>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>18640.94</t>
+          <t>27177.70</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>62397.56</t>
+          <t>637.84</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>18630.91</t>
+          <t/>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>72836.22</t>
+          <t>637.84</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>199108.89</t>
+          <t>27177.70</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1483,22 +1483,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11062.00</t>
+          <t/>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>182802.61</t>
+          <t/>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>173344.11</t>
+          <t>801.50</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>185870.02</t>
+          <t/>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>15917.48</t>
+          <t>11081.00</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>18466.20</t>
+          <t>4856.33</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>63423.28</t>
+          <t>168090.51</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>18438.28</t>
+          <t/>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>263746.87</t>
+          <t>179973.01</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>405577.11</t>
+          <t>4856.33</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1585,17 +1585,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>153436.60</t>
+          <t/>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>4847.30</t>
+          <t/>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>22.09</t>
+          <t/>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1605,14 +1605,14 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>3752.34</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>13.05</t>
-        </is>
-      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t/>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>57932.67</t>
+          <t/>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1635,12 +1635,12 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>66532.31</t>
+          <t/>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>153471.74</t>
+          <t>3752.34</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1682,17 +1682,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>102207.65</t>
+          <t/>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5604.27</t>
+          <t/>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2517.11</t>
+          <t/>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1702,12 +1702,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4509.31</t>
+          <t/>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2504.06</t>
+          <t>6947.38</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1717,12 +1717,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16188.23</t>
+          <t>9985.47</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2494.00</t>
+          <t/>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>26301.81</t>
+          <t>9985.47</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>109722.82</t>
+          <t>6947.38</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1779,42 +1779,42 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>54103.70</t>
+          <t/>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3165.27</t>
+          <t>30000.00</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>29.13</t>
+          <t>5.20</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t/>
+          <t>2494.00</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2352.89</t>
+          <t>23263.84</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>18.07</t>
+          <t>2358.09</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t/>
+          <t>2494.00</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>59695.25</t>
+          <t>5323.90</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1829,17 +1829,17 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>65213.41</t>
+          <t>58587.74</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>54150.90</t>
+          <t>2363.29</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t/>
+          <t>4988.00</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">

</xml_diff>

<commit_message>
Improve tax and operating cost validation accuracy
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/monthly_cash_flow_reconstruction.xlsx
+++ b/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/monthly_cash_flow_reconstruction.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>68868.69</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>137737.38</t>
+          <t>68888.69</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1809,37 +1809,37 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>5323.90</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>58587.74</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2363.29</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
           <t>2494.00</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>5323.90</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>58587.74</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>2363.29</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>4988.00</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">

</xml_diff>